<commit_message>
Player spawn fixed, bug fixed of bags falling trough the map.
</commit_message>
<xml_diff>
--- a/Prog4Game/Data/Levels/Level_Editor.xlsx
+++ b/Prog4Game/Data/Levels/Level_Editor.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DAE\GD-Y2\Programming4\Assignments\Project\Prog4-Engine\Prog4Game\Data\Levels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C3F861D-828A-4FF1-983C-1EF2A65E6C4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{678E9E4A-DBB7-4DF5-A103-4F22EAAAD2C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="13776" xr2:uid="{249B810F-626A-4F90-9DE6-B7EB3113683C}"/>
+    <workbookView xWindow="3204" yWindow="4116" windowWidth="18132" windowHeight="9564" activeTab="2" xr2:uid="{249B810F-626A-4F90-9DE6-B7EB3113683C}"/>
   </bookViews>
   <sheets>
     <sheet name="LVL_00" sheetId="1" r:id="rId1"/>
@@ -77,11 +77,18 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="18">
+  <dxfs count="15">
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFC000"/>
+          <bgColor theme="1" tint="0.34998626667073579"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="-0.24994659260841701"/>
         </patternFill>
       </fill>
     </dxf>
@@ -95,20 +102,6 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="5" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="0.34998626667073579"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
           <bgColor rgb="FFFFC000"/>
         </patternFill>
       </fill>
@@ -116,49 +109,7 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="0.34998626667073579"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="0.34998626667073579"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
+          <bgColor rgb="FF0070C0"/>
         </patternFill>
       </fill>
     </dxf>
@@ -186,7 +137,14 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="5" tint="-0.24994659260841701"/>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0070C0"/>
         </patternFill>
       </fill>
     </dxf>
@@ -200,7 +158,28 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="1" tint="0.34998626667073579"/>
+          <bgColor theme="5" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0070C0"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1012,17 +991,20 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A1:O10">
-    <cfRule type="containsText" dxfId="12" priority="4" operator="containsText" text="0">
-      <formula>NOT(ISERROR(SEARCH("0",A1)))</formula>
+    <cfRule type="containsText" dxfId="14" priority="1" operator="containsText" text="5">
+      <formula>NOT(ISERROR(SEARCH("5",A1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="13" priority="3" operator="containsText" text="1">
+    <cfRule type="containsText" dxfId="13" priority="2" operator="containsText" text="3">
+      <formula>NOT(ISERROR(SEARCH("3",A1)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="12" priority="3" operator="containsText" text="2">
+      <formula>NOT(ISERROR(SEARCH("2",A1)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="11" priority="4" operator="containsText" text="1">
       <formula>NOT(ISERROR(SEARCH("1",A1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="14" priority="2" operator="containsText" text="2">
-      <formula>NOT(ISERROR(SEARCH("2",A1)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="11" priority="1" operator="containsText" text="3">
-      <formula>NOT(ISERROR(SEARCH("3",A1)))</formula>
+    <cfRule type="containsText" dxfId="10" priority="5" operator="containsText" text="0">
+      <formula>NOT(ISERROR(SEARCH("0",A1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1510,16 +1492,19 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A1:O10">
-    <cfRule type="containsText" dxfId="4" priority="1" operator="containsText" text="3">
+    <cfRule type="containsText" dxfId="9" priority="1" operator="containsText" text="5">
+      <formula>NOT(ISERROR(SEARCH("5",A1)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="8" priority="2" operator="containsText" text="3">
       <formula>NOT(ISERROR(SEARCH("3",A1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="5" priority="2" operator="containsText" text="2">
+    <cfRule type="containsText" dxfId="7" priority="3" operator="containsText" text="2">
       <formula>NOT(ISERROR(SEARCH("2",A1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="6" priority="3" operator="containsText" text="1">
+    <cfRule type="containsText" dxfId="6" priority="4" operator="containsText" text="1">
       <formula>NOT(ISERROR(SEARCH("1",A1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="7" priority="4" operator="containsText" text="0">
+    <cfRule type="containsText" dxfId="5" priority="5" operator="containsText" text="0">
       <formula>NOT(ISERROR(SEARCH("0",A1)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2007,16 +1992,19 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A1:O10">
-    <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="3">
+    <cfRule type="containsText" dxfId="4" priority="1" operator="containsText" text="5">
+      <formula>NOT(ISERROR(SEARCH("5",A1)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="3" priority="2" operator="containsText" text="3">
       <formula>NOT(ISERROR(SEARCH("3",A1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="2">
+    <cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="2">
       <formula>NOT(ISERROR(SEARCH("2",A1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="1">
+    <cfRule type="containsText" dxfId="1" priority="4" operator="containsText" text="1">
       <formula>NOT(ISERROR(SEARCH("1",A1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="0">
+    <cfRule type="containsText" dxfId="0" priority="5" operator="containsText" text="0">
       <formula>NOT(ISERROR(SEARCH("0",A1)))</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Added audio back in, tried scene swapping [Broken only works sometimes]
</commit_message>
<xml_diff>
--- a/Prog4Game/Data/Levels/Level_Editor.xlsx
+++ b/Prog4Game/Data/Levels/Level_Editor.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DAE\GD-Y2\Programming4\Assignments\Project\Prog4-Engine\Prog4Game\Data\Levels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{678E9E4A-DBB7-4DF5-A103-4F22EAAAD2C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6122BD51-E853-4594-9784-AAAAE0A46B83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3204" yWindow="4116" windowWidth="18132" windowHeight="9564" activeTab="2" xr2:uid="{249B810F-626A-4F90-9DE6-B7EB3113683C}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="13776" activeTab="2" xr2:uid="{249B810F-626A-4F90-9DE6-B7EB3113683C}"/>
   </bookViews>
   <sheets>
     <sheet name="LVL_00" sheetId="1" r:id="rId1"/>
@@ -1025,40 +1025,40 @@
         <v>0</v>
       </c>
       <c r="B1" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C1" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D1" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E1" s="1">
+        <v>0</v>
+      </c>
+      <c r="F1" s="1">
+        <v>0</v>
+      </c>
+      <c r="G1" s="1">
+        <v>1</v>
+      </c>
+      <c r="H1" s="1">
+        <v>1</v>
+      </c>
+      <c r="I1" s="1">
         <v>3</v>
       </c>
-      <c r="F1" s="1">
-        <v>1</v>
-      </c>
-      <c r="G1" s="1">
-        <v>1</v>
-      </c>
-      <c r="H1" s="1">
-        <v>1</v>
-      </c>
-      <c r="I1" s="1">
-        <v>1</v>
-      </c>
       <c r="J1" s="1">
         <v>1</v>
       </c>
       <c r="K1" s="1">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L1" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M1" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N1" s="1">
         <v>0</v>
@@ -1069,31 +1069,531 @@
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B2" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C2" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D2" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E2" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F2" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G2" s="1">
         <v>1</v>
       </c>
       <c r="H2" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I2" s="1">
         <v>1</v>
+      </c>
+      <c r="J2" s="1">
+        <v>1</v>
+      </c>
+      <c r="K2" s="1">
+        <v>2</v>
+      </c>
+      <c r="L2" s="1">
+        <v>1</v>
+      </c>
+      <c r="M2" s="1">
+        <v>1</v>
+      </c>
+      <c r="N2" s="1">
+        <v>0</v>
+      </c>
+      <c r="O2" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A3" s="1">
+        <v>1</v>
+      </c>
+      <c r="B3" s="1">
+        <v>2</v>
+      </c>
+      <c r="C3" s="1">
+        <v>2</v>
+      </c>
+      <c r="D3" s="1">
+        <v>1</v>
+      </c>
+      <c r="E3" s="1">
+        <v>1</v>
+      </c>
+      <c r="F3" s="1">
+        <v>0</v>
+      </c>
+      <c r="G3" s="1">
+        <v>1</v>
+      </c>
+      <c r="H3" s="1">
+        <v>2</v>
+      </c>
+      <c r="I3" s="1">
+        <v>2</v>
+      </c>
+      <c r="J3" s="1">
+        <v>2</v>
+      </c>
+      <c r="K3" s="1">
+        <v>2</v>
+      </c>
+      <c r="L3" s="1">
+        <v>2</v>
+      </c>
+      <c r="M3" s="1">
+        <v>1</v>
+      </c>
+      <c r="N3" s="1">
+        <v>0</v>
+      </c>
+      <c r="O3" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A4" s="1">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1">
+        <v>2</v>
+      </c>
+      <c r="C4" s="1">
+        <v>2</v>
+      </c>
+      <c r="D4" s="1">
+        <v>3</v>
+      </c>
+      <c r="E4" s="1">
+        <v>1</v>
+      </c>
+      <c r="F4" s="1">
+        <v>0</v>
+      </c>
+      <c r="G4" s="1">
+        <v>1</v>
+      </c>
+      <c r="H4" s="1">
+        <v>2</v>
+      </c>
+      <c r="I4" s="1">
+        <v>2</v>
+      </c>
+      <c r="J4" s="1">
+        <v>2</v>
+      </c>
+      <c r="K4" s="1">
+        <v>2</v>
+      </c>
+      <c r="L4" s="1">
+        <v>2</v>
+      </c>
+      <c r="M4" s="1">
+        <v>1</v>
+      </c>
+      <c r="N4" s="1">
+        <v>0</v>
+      </c>
+      <c r="O4" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A5" s="1">
+        <v>2</v>
+      </c>
+      <c r="B5" s="1">
+        <v>2</v>
+      </c>
+      <c r="C5" s="1">
+        <v>2</v>
+      </c>
+      <c r="D5" s="1">
+        <v>2</v>
+      </c>
+      <c r="E5" s="1">
+        <v>1</v>
+      </c>
+      <c r="F5" s="1">
+        <v>0</v>
+      </c>
+      <c r="G5" s="1">
+        <v>1</v>
+      </c>
+      <c r="H5" s="1">
+        <v>1</v>
+      </c>
+      <c r="I5" s="1">
+        <v>1</v>
+      </c>
+      <c r="J5" s="1">
+        <v>1</v>
+      </c>
+      <c r="K5" s="1">
+        <v>1</v>
+      </c>
+      <c r="L5" s="1">
+        <v>1</v>
+      </c>
+      <c r="M5" s="1">
+        <v>1</v>
+      </c>
+      <c r="N5" s="1">
+        <v>0</v>
+      </c>
+      <c r="O5" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A6" s="1">
+        <v>2</v>
+      </c>
+      <c r="B6" s="1">
+        <v>2</v>
+      </c>
+      <c r="C6" s="1">
+        <v>2</v>
+      </c>
+      <c r="D6" s="1">
+        <v>2</v>
+      </c>
+      <c r="E6" s="1">
+        <v>1</v>
+      </c>
+      <c r="F6" s="1">
+        <v>0</v>
+      </c>
+      <c r="G6" s="1">
+        <v>1</v>
+      </c>
+      <c r="H6" s="1">
+        <v>3</v>
+      </c>
+      <c r="I6" s="1">
+        <v>1</v>
+      </c>
+      <c r="J6" s="1">
+        <v>1</v>
+      </c>
+      <c r="K6" s="1">
+        <v>0</v>
+      </c>
+      <c r="L6" s="1">
+        <v>0</v>
+      </c>
+      <c r="M6" s="1">
+        <v>0</v>
+      </c>
+      <c r="N6" s="1">
+        <v>0</v>
+      </c>
+      <c r="O6" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A7" s="1">
+        <v>1</v>
+      </c>
+      <c r="B7" s="1">
+        <v>2</v>
+      </c>
+      <c r="C7" s="1">
+        <v>2</v>
+      </c>
+      <c r="D7" s="1">
+        <v>1</v>
+      </c>
+      <c r="E7" s="1">
+        <v>1</v>
+      </c>
+      <c r="F7" s="1">
+        <v>0</v>
+      </c>
+      <c r="G7" s="1">
+        <v>1</v>
+      </c>
+      <c r="H7" s="1">
+        <v>2</v>
+      </c>
+      <c r="I7" s="1">
+        <v>2</v>
+      </c>
+      <c r="J7" s="1">
+        <v>1</v>
+      </c>
+      <c r="K7" s="1">
+        <v>0</v>
+      </c>
+      <c r="L7" s="1">
+        <v>1</v>
+      </c>
+      <c r="M7" s="1">
+        <v>1</v>
+      </c>
+      <c r="N7" s="1">
+        <v>1</v>
+      </c>
+      <c r="O7" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A8" s="1">
+        <v>1</v>
+      </c>
+      <c r="B8" s="1">
+        <v>3</v>
+      </c>
+      <c r="C8" s="1">
+        <v>3</v>
+      </c>
+      <c r="D8" s="1">
+        <v>1</v>
+      </c>
+      <c r="E8" s="1">
+        <v>1</v>
+      </c>
+      <c r="F8" s="1">
+        <v>0</v>
+      </c>
+      <c r="G8" s="1">
+        <v>2</v>
+      </c>
+      <c r="H8" s="1">
+        <v>2</v>
+      </c>
+      <c r="I8" s="1">
+        <v>2</v>
+      </c>
+      <c r="J8" s="1">
+        <v>2</v>
+      </c>
+      <c r="K8" s="1">
+        <v>0</v>
+      </c>
+      <c r="L8" s="1">
+        <v>1</v>
+      </c>
+      <c r="M8" s="1">
+        <v>2</v>
+      </c>
+      <c r="N8" s="1">
+        <v>2</v>
+      </c>
+      <c r="O8" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A9" s="1">
+        <v>2</v>
+      </c>
+      <c r="B9" s="1">
+        <v>1</v>
+      </c>
+      <c r="C9" s="1">
+        <v>1</v>
+      </c>
+      <c r="D9" s="1">
+        <v>1</v>
+      </c>
+      <c r="E9" s="1">
+        <v>1</v>
+      </c>
+      <c r="F9" s="1">
+        <v>0</v>
+      </c>
+      <c r="G9" s="1">
+        <v>1</v>
+      </c>
+      <c r="H9" s="1">
+        <v>2</v>
+      </c>
+      <c r="I9" s="1">
+        <v>2</v>
+      </c>
+      <c r="J9" s="1">
+        <v>1</v>
+      </c>
+      <c r="K9" s="1">
+        <v>0</v>
+      </c>
+      <c r="L9" s="1">
+        <v>1</v>
+      </c>
+      <c r="M9" s="1">
+        <v>2</v>
+      </c>
+      <c r="N9" s="1">
+        <v>2</v>
+      </c>
+      <c r="O9" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A10" s="1">
+        <v>2</v>
+      </c>
+      <c r="B10" s="1">
+        <v>2</v>
+      </c>
+      <c r="C10" s="1">
+        <v>1</v>
+      </c>
+      <c r="D10" s="1">
+        <v>1</v>
+      </c>
+      <c r="E10" s="1">
+        <v>1</v>
+      </c>
+      <c r="F10" s="1">
+        <v>0</v>
+      </c>
+      <c r="G10" s="1">
+        <v>0</v>
+      </c>
+      <c r="H10" s="1">
+        <v>0</v>
+      </c>
+      <c r="I10" s="1">
+        <v>0</v>
+      </c>
+      <c r="J10" s="1">
+        <v>0</v>
+      </c>
+      <c r="K10" s="1">
+        <v>0</v>
+      </c>
+      <c r="L10" s="1">
+        <v>1</v>
+      </c>
+      <c r="M10" s="1">
+        <v>1</v>
+      </c>
+      <c r="N10" s="1">
+        <v>1</v>
+      </c>
+      <c r="O10" s="1">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="A1:O10">
+    <cfRule type="containsText" dxfId="4" priority="1" operator="containsText" text="5">
+      <formula>NOT(ISERROR(SEARCH("5",A1)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="3" priority="2" operator="containsText" text="3">
+      <formula>NOT(ISERROR(SEARCH("3",A1)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="2">
+      <formula>NOT(ISERROR(SEARCH("2",A1)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="1" priority="4" operator="containsText" text="1">
+      <formula>NOT(ISERROR(SEARCH("1",A1)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="0" priority="5" operator="containsText" text="0">
+      <formula>NOT(ISERROR(SEARCH("0",A1)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA2784A3-F880-40FE-9D8D-DF50A2747251}">
+  <dimension ref="A1:O10"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="15" width="4.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A1" s="1">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1">
+        <v>0</v>
+      </c>
+      <c r="D1" s="1">
+        <v>0</v>
+      </c>
+      <c r="E1" s="1">
+        <v>0</v>
+      </c>
+      <c r="F1" s="1">
+        <v>3</v>
+      </c>
+      <c r="G1" s="1">
+        <v>1</v>
+      </c>
+      <c r="H1" s="1">
+        <v>3</v>
+      </c>
+      <c r="I1" s="1">
+        <v>1</v>
+      </c>
+      <c r="J1" s="1">
+        <v>3</v>
+      </c>
+      <c r="K1" s="1">
+        <v>0</v>
+      </c>
+      <c r="L1" s="1">
+        <v>0</v>
+      </c>
+      <c r="M1" s="1">
+        <v>0</v>
+      </c>
+      <c r="N1" s="1">
+        <v>0</v>
+      </c>
+      <c r="O1" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A2" s="1">
+        <v>2</v>
+      </c>
+      <c r="B2" s="1">
+        <v>2</v>
+      </c>
+      <c r="C2" s="1">
+        <v>1</v>
+      </c>
+      <c r="D2" s="1">
+        <v>1</v>
+      </c>
+      <c r="E2" s="1">
+        <v>0</v>
+      </c>
+      <c r="F2" s="1">
+        <v>1</v>
+      </c>
+      <c r="G2" s="1">
+        <v>2</v>
+      </c>
+      <c r="H2" s="1">
+        <v>1</v>
+      </c>
+      <c r="I2" s="1">
+        <v>2</v>
       </c>
       <c r="J2" s="1">
         <v>1</v>
@@ -1108,7 +1608,7 @@
         <v>3</v>
       </c>
       <c r="N2" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O2" s="1">
         <v>1</v>
@@ -1116,31 +1616,31 @@
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B3" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C3" s="1">
         <v>1</v>
       </c>
       <c r="D3" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E3" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F3" s="1">
         <v>1</v>
       </c>
       <c r="G3" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H3" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I3" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J3" s="1">
         <v>1</v>
@@ -1152,10 +1652,10 @@
         <v>1</v>
       </c>
       <c r="M3" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N3" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O3" s="1">
         <v>1</v>
@@ -1163,31 +1663,31 @@
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B4" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C4" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D4" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E4" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F4" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G4" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H4" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I4" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J4" s="1">
         <v>1</v>
@@ -1196,7 +1696,7 @@
         <v>0</v>
       </c>
       <c r="L4" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M4" s="1">
         <v>2</v>
@@ -1210,31 +1710,31 @@
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B5" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C5" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D5" s="1">
         <v>2</v>
       </c>
       <c r="E5" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F5" s="1">
         <v>1</v>
       </c>
       <c r="G5" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H5" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I5" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J5" s="1">
         <v>1</v>
@@ -1243,7 +1743,7 @@
         <v>0</v>
       </c>
       <c r="L5" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M5" s="1">
         <v>2</v>
@@ -1257,34 +1757,34 @@
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B6" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C6" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D6" s="1">
         <v>2</v>
       </c>
       <c r="E6" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F6" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G6" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H6" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I6" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J6" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K6" s="1">
         <v>0</v>
@@ -1299,7 +1799,7 @@
         <v>2</v>
       </c>
       <c r="O6" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.3">
@@ -1307,10 +1807,10 @@
         <v>1</v>
       </c>
       <c r="B7" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C7" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D7" s="1">
         <v>1</v>
@@ -1319,31 +1819,31 @@
         <v>1</v>
       </c>
       <c r="F7" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G7" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H7" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I7" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J7" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K7" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L7" s="1">
         <v>1</v>
       </c>
       <c r="M7" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N7" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O7" s="1">
         <v>1</v>
@@ -1354,34 +1854,34 @@
         <v>1</v>
       </c>
       <c r="B8" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C8" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D8" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E8" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F8" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G8" s="1">
         <v>1</v>
       </c>
       <c r="H8" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I8" s="1">
         <v>1</v>
       </c>
       <c r="J8" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K8" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L8" s="1">
         <v>1</v>
@@ -1410,25 +1910,25 @@
         <v>1</v>
       </c>
       <c r="E9" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F9" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G9" s="1">
         <v>1</v>
       </c>
       <c r="H9" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I9" s="1">
         <v>1</v>
       </c>
       <c r="J9" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K9" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L9" s="1">
         <v>1</v>
@@ -1457,25 +1957,25 @@
         <v>1</v>
       </c>
       <c r="E10" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F10" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G10" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H10" s="1">
         <v>0</v>
       </c>
       <c r="I10" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J10" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K10" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L10" s="1">
         <v>1</v>
@@ -1510,504 +2010,4 @@
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA2784A3-F880-40FE-9D8D-DF50A2747251}">
-  <dimension ref="A1:O10"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="15" width="4.77734375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A1" s="1">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1">
-        <v>1</v>
-      </c>
-      <c r="D1" s="1">
-        <v>1</v>
-      </c>
-      <c r="E1" s="1">
-        <v>3</v>
-      </c>
-      <c r="F1" s="1">
-        <v>1</v>
-      </c>
-      <c r="G1" s="1">
-        <v>1</v>
-      </c>
-      <c r="H1" s="1">
-        <v>1</v>
-      </c>
-      <c r="I1" s="1">
-        <v>1</v>
-      </c>
-      <c r="J1" s="1">
-        <v>1</v>
-      </c>
-      <c r="K1" s="1">
-        <v>0</v>
-      </c>
-      <c r="L1" s="1">
-        <v>0</v>
-      </c>
-      <c r="M1" s="1">
-        <v>0</v>
-      </c>
-      <c r="N1" s="1">
-        <v>0</v>
-      </c>
-      <c r="O1" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A2" s="1">
-        <v>0</v>
-      </c>
-      <c r="B2" s="1">
-        <v>1</v>
-      </c>
-      <c r="C2" s="1">
-        <v>1</v>
-      </c>
-      <c r="D2" s="1">
-        <v>2</v>
-      </c>
-      <c r="E2" s="1">
-        <v>2</v>
-      </c>
-      <c r="F2" s="1">
-        <v>1</v>
-      </c>
-      <c r="G2" s="1">
-        <v>1</v>
-      </c>
-      <c r="H2" s="1">
-        <v>2</v>
-      </c>
-      <c r="I2" s="1">
-        <v>1</v>
-      </c>
-      <c r="J2" s="1">
-        <v>1</v>
-      </c>
-      <c r="K2" s="1">
-        <v>0</v>
-      </c>
-      <c r="L2" s="1">
-        <v>1</v>
-      </c>
-      <c r="M2" s="1">
-        <v>3</v>
-      </c>
-      <c r="N2" s="1">
-        <v>1</v>
-      </c>
-      <c r="O2" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A3" s="1">
-        <v>0</v>
-      </c>
-      <c r="B3" s="1">
-        <v>3</v>
-      </c>
-      <c r="C3" s="1">
-        <v>1</v>
-      </c>
-      <c r="D3" s="1">
-        <v>2</v>
-      </c>
-      <c r="E3" s="1">
-        <v>2</v>
-      </c>
-      <c r="F3" s="1">
-        <v>1</v>
-      </c>
-      <c r="G3" s="1">
-        <v>1</v>
-      </c>
-      <c r="H3" s="1">
-        <v>2</v>
-      </c>
-      <c r="I3" s="1">
-        <v>1</v>
-      </c>
-      <c r="J3" s="1">
-        <v>1</v>
-      </c>
-      <c r="K3" s="1">
-        <v>0</v>
-      </c>
-      <c r="L3" s="1">
-        <v>1</v>
-      </c>
-      <c r="M3" s="1">
-        <v>1</v>
-      </c>
-      <c r="N3" s="1">
-        <v>1</v>
-      </c>
-      <c r="O3" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A4" s="1">
-        <v>0</v>
-      </c>
-      <c r="B4" s="1">
-        <v>1</v>
-      </c>
-      <c r="C4" s="1">
-        <v>1</v>
-      </c>
-      <c r="D4" s="1">
-        <v>2</v>
-      </c>
-      <c r="E4" s="1">
-        <v>2</v>
-      </c>
-      <c r="F4" s="1">
-        <v>3</v>
-      </c>
-      <c r="G4" s="1">
-        <v>1</v>
-      </c>
-      <c r="H4" s="1">
-        <v>2</v>
-      </c>
-      <c r="I4" s="1">
-        <v>3</v>
-      </c>
-      <c r="J4" s="1">
-        <v>1</v>
-      </c>
-      <c r="K4" s="1">
-        <v>0</v>
-      </c>
-      <c r="L4" s="1">
-        <v>1</v>
-      </c>
-      <c r="M4" s="1">
-        <v>2</v>
-      </c>
-      <c r="N4" s="1">
-        <v>2</v>
-      </c>
-      <c r="O4" s="1">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A5" s="1">
-        <v>0</v>
-      </c>
-      <c r="B5" s="1">
-        <v>1</v>
-      </c>
-      <c r="C5" s="1">
-        <v>1</v>
-      </c>
-      <c r="D5" s="1">
-        <v>2</v>
-      </c>
-      <c r="E5" s="1">
-        <v>2</v>
-      </c>
-      <c r="F5" s="1">
-        <v>1</v>
-      </c>
-      <c r="G5" s="1">
-        <v>1</v>
-      </c>
-      <c r="H5" s="1">
-        <v>2</v>
-      </c>
-      <c r="I5" s="1">
-        <v>1</v>
-      </c>
-      <c r="J5" s="1">
-        <v>1</v>
-      </c>
-      <c r="K5" s="1">
-        <v>0</v>
-      </c>
-      <c r="L5" s="1">
-        <v>1</v>
-      </c>
-      <c r="M5" s="1">
-        <v>2</v>
-      </c>
-      <c r="N5" s="1">
-        <v>2</v>
-      </c>
-      <c r="O5" s="1">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A6" s="1">
-        <v>0</v>
-      </c>
-      <c r="B6" s="1">
-        <v>0</v>
-      </c>
-      <c r="C6" s="1">
-        <v>1</v>
-      </c>
-      <c r="D6" s="1">
-        <v>2</v>
-      </c>
-      <c r="E6" s="1">
-        <v>2</v>
-      </c>
-      <c r="F6" s="1">
-        <v>1</v>
-      </c>
-      <c r="G6" s="1">
-        <v>1</v>
-      </c>
-      <c r="H6" s="1">
-        <v>2</v>
-      </c>
-      <c r="I6" s="1">
-        <v>1</v>
-      </c>
-      <c r="J6" s="1">
-        <v>1</v>
-      </c>
-      <c r="K6" s="1">
-        <v>0</v>
-      </c>
-      <c r="L6" s="1">
-        <v>1</v>
-      </c>
-      <c r="M6" s="1">
-        <v>2</v>
-      </c>
-      <c r="N6" s="1">
-        <v>2</v>
-      </c>
-      <c r="O6" s="1">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A7" s="1">
-        <v>1</v>
-      </c>
-      <c r="B7" s="1">
-        <v>0</v>
-      </c>
-      <c r="C7" s="1">
-        <v>1</v>
-      </c>
-      <c r="D7" s="1">
-        <v>1</v>
-      </c>
-      <c r="E7" s="1">
-        <v>1</v>
-      </c>
-      <c r="F7" s="1">
-        <v>1</v>
-      </c>
-      <c r="G7" s="1">
-        <v>3</v>
-      </c>
-      <c r="H7" s="1">
-        <v>1</v>
-      </c>
-      <c r="I7" s="1">
-        <v>3</v>
-      </c>
-      <c r="J7" s="1">
-        <v>1</v>
-      </c>
-      <c r="K7" s="1">
-        <v>0</v>
-      </c>
-      <c r="L7" s="1">
-        <v>1</v>
-      </c>
-      <c r="M7" s="1">
-        <v>1</v>
-      </c>
-      <c r="N7" s="1">
-        <v>1</v>
-      </c>
-      <c r="O7" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A8" s="1">
-        <v>1</v>
-      </c>
-      <c r="B8" s="1">
-        <v>0</v>
-      </c>
-      <c r="C8" s="1">
-        <v>0</v>
-      </c>
-      <c r="D8" s="1">
-        <v>0</v>
-      </c>
-      <c r="E8" s="1">
-        <v>0</v>
-      </c>
-      <c r="F8" s="1">
-        <v>1</v>
-      </c>
-      <c r="G8" s="1">
-        <v>1</v>
-      </c>
-      <c r="H8" s="1">
-        <v>1</v>
-      </c>
-      <c r="I8" s="1">
-        <v>1</v>
-      </c>
-      <c r="J8" s="1">
-        <v>1</v>
-      </c>
-      <c r="K8" s="1">
-        <v>0</v>
-      </c>
-      <c r="L8" s="1">
-        <v>1</v>
-      </c>
-      <c r="M8" s="1">
-        <v>1</v>
-      </c>
-      <c r="N8" s="1">
-        <v>1</v>
-      </c>
-      <c r="O8" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A9" s="1">
-        <v>2</v>
-      </c>
-      <c r="B9" s="1">
-        <v>1</v>
-      </c>
-      <c r="C9" s="1">
-        <v>1</v>
-      </c>
-      <c r="D9" s="1">
-        <v>1</v>
-      </c>
-      <c r="E9" s="1">
-        <v>0</v>
-      </c>
-      <c r="F9" s="1">
-        <v>1</v>
-      </c>
-      <c r="G9" s="1">
-        <v>1</v>
-      </c>
-      <c r="H9" s="1">
-        <v>1</v>
-      </c>
-      <c r="I9" s="1">
-        <v>1</v>
-      </c>
-      <c r="J9" s="1">
-        <v>1</v>
-      </c>
-      <c r="K9" s="1">
-        <v>0</v>
-      </c>
-      <c r="L9" s="1">
-        <v>1</v>
-      </c>
-      <c r="M9" s="1">
-        <v>1</v>
-      </c>
-      <c r="N9" s="1">
-        <v>1</v>
-      </c>
-      <c r="O9" s="1">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A10" s="1">
-        <v>2</v>
-      </c>
-      <c r="B10" s="1">
-        <v>2</v>
-      </c>
-      <c r="C10" s="1">
-        <v>1</v>
-      </c>
-      <c r="D10" s="1">
-        <v>1</v>
-      </c>
-      <c r="E10" s="1">
-        <v>0</v>
-      </c>
-      <c r="F10" s="1">
-        <v>0</v>
-      </c>
-      <c r="G10" s="1">
-        <v>0</v>
-      </c>
-      <c r="H10" s="1">
-        <v>0</v>
-      </c>
-      <c r="I10" s="1">
-        <v>0</v>
-      </c>
-      <c r="J10" s="1">
-        <v>0</v>
-      </c>
-      <c r="K10" s="1">
-        <v>0</v>
-      </c>
-      <c r="L10" s="1">
-        <v>1</v>
-      </c>
-      <c r="M10" s="1">
-        <v>1</v>
-      </c>
-      <c r="N10" s="1">
-        <v>2</v>
-      </c>
-      <c r="O10" s="1">
-        <v>2</v>
-      </c>
-    </row>
-  </sheetData>
-  <conditionalFormatting sqref="A1:O10">
-    <cfRule type="containsText" dxfId="4" priority="1" operator="containsText" text="5">
-      <formula>NOT(ISERROR(SEARCH("5",A1)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="3" priority="2" operator="containsText" text="3">
-      <formula>NOT(ISERROR(SEARCH("3",A1)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="2">
-      <formula>NOT(ISERROR(SEARCH("2",A1)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="1" priority="4" operator="containsText" text="1">
-      <formula>NOT(ISERROR(SEARCH("1",A1)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="0" priority="5" operator="containsText" text="0">
-      <formula>NOT(ISERROR(SEARCH("0",A1)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>